<commit_message>
Refresh QR code module v1.20 and scanner UX
Refresh the QR/barcode capability to the v1.20 Master Book contract. This update modernizes the native scanner experience, keeps the canonical barcode output contract intact, updates method metadata (version, maturity, connectivity, and discovery fields), and refreshes the ODK XLSForm examples and documentation. It also removes stale generated XML projections and records the validation status for the refreshed scanner flow.
</commit_message>
<xml_diff>
--- a/app/src/main/assets/methodmesh/odk_templates/qrcode/example_odk_barcode_scan.xlsx
+++ b/app/src/main/assets/methodmesh/odk_templates/qrcode/example_odk_barcode_scan.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R1738ea4c69274ff2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R651fe5e9794d4d90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R63ff11fe72d74ba9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R99ce503f971341d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R01cb83a4c40c4016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rb55017c9e7e9476f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -365,309 +365,443 @@
         <x:v>label</x:v>
       </x:c>
       <x:c r="D1" t="str">
+        <x:v>hint</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
         <x:v>appearance</x:v>
       </x:c>
-      <x:c r="E1" t="str">
+      <x:c r="F1" t="str">
+        <x:v>required</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>relevant</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>constraint</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>constraint_message</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>calculation</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>default</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>read_only</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
         <x:v>body::intent</x:v>
-      </x:c>
-      <x:c r="F1" t="str">
-        <x:v>calculation</x:v>
-      </x:c>
-      <x:c r="G1" t="str">
-        <x:v>required</x:v>
-      </x:c>
-      <x:c r="H1" t="str">
-        <x:v>readonly</x:v>
-      </x:c>
-      <x:c r="I1" t="str">
-        <x:v>relevant</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>select_multiple barcode_format</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>barcode_formats_input</x:v>
+        <x:v>intro</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Accepted code formats (optional)</x:v>
-      </x:c>
-      <x:c r="D2"/>
+        <x:v>MethodMesh Automatic code scanner — barcode.scan</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>Scan a QR, Data Matrix, Aztec, PDF417 or common 1D barcode with MethodMesh. The scan is performed in the native scanner and returned only after Commit.</x:v>
+      </x:c>
       <x:c r="E2"/>
       <x:c r="F2"/>
       <x:c r="G2"/>
       <x:c r="H2"/>
       <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
+      <x:c r="M2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
         <x:v>begin_group</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>code_scan</x:v>
+        <x:v>run_barcode_scan</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Scan code</x:v>
+        <x:v>Run barcode.scan</x:v>
       </x:c>
       <x:c r="D3" t="str">
+        <x:v>One MethodMesh capability invocation. Canonical return fields are unprefixed and the shared metadata payload is captured in methodmesh_full_json.</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
         <x:v>field-list</x:v>
-      </x:c>
-      <x:c r="E3" t="str">
-        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='barcode.scan',input_barcode_formats=${barcode_formats_input},input_payload_mode='FULL',methodmesh_return_namespace='scan',return_mode='flat')</x:v>
       </x:c>
       <x:c r="F3"/>
       <x:c r="G3"/>
       <x:c r="H3"/>
       <x:c r="I3"/>
+      <x:c r="J3"/>
+      <x:c r="K3"/>
+      <x:c r="L3"/>
+      <x:c r="M3" t="str">
+        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='barcode.scan',input_barcode_formats=${barcode_formats_input},input_payload_mode='FULL',return_mode='flat')</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>text</x:v>
+        <x:v>select_multiple barcode_format</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>scan_methodmesh_execution_id</x:v>
+        <x:v>barcode_formats_input</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>MethodMesh execution ID</x:v>
-      </x:c>
-      <x:c r="D4"/>
+        <x:v>Accepted code formats (optional)</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Leave blank for automatic detection of all supported formats.</x:v>
+      </x:c>
       <x:c r="E4"/>
       <x:c r="F4"/>
       <x:c r="G4"/>
-      <x:c r="H4" t="str">
-        <x:v>yes</x:v>
-      </x:c>
+      <x:c r="H4"/>
       <x:c r="I4"/>
+      <x:c r="J4"/>
+      <x:c r="K4"/>
+      <x:c r="L4"/>
+      <x:c r="M4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>scan_methodmesh_status</x:v>
+        <x:v>methodmesh_status</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>MethodMesh status</x:v>
       </x:c>
-      <x:c r="D5"/>
-      <x:c r="E5"/>
+      <x:c r="D5" t="str">
+        <x:v>Shared MethodMesh transport status.</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F5"/>
       <x:c r="G5"/>
-      <x:c r="H5" t="str">
+      <x:c r="H5"/>
+      <x:c r="I5"/>
+      <x:c r="J5"/>
+      <x:c r="K5"/>
+      <x:c r="L5" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="I5"/>
+      <x:c r="M5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>scan_barcode_payload</x:v>
+        <x:v>barcode_payload</x:v>
       </x:c>
       <x:c r="C6" t="str">
         <x:v>Decoded payload</x:v>
       </x:c>
-      <x:c r="D6"/>
-      <x:c r="E6"/>
+      <x:c r="D6" t="str">
+        <x:v>Primary barcode.scan result.</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F6"/>
-      <x:c r="G6" t="str">
+      <x:c r="G6"/>
+      <x:c r="H6"/>
+      <x:c r="I6"/>
+      <x:c r="J6"/>
+      <x:c r="K6"/>
+      <x:c r="L6" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="H6" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="I6"/>
+      <x:c r="M6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>scan_barcode_format</x:v>
+        <x:v>barcode_format</x:v>
       </x:c>
       <x:c r="C7" t="str">
         <x:v>Detected barcode format</x:v>
       </x:c>
-      <x:c r="D7"/>
-      <x:c r="E7"/>
+      <x:c r="D7" t="str">
+        <x:v>Canonical barcode format name.</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F7"/>
       <x:c r="G7"/>
-      <x:c r="H7" t="str">
+      <x:c r="H7"/>
+      <x:c r="I7"/>
+      <x:c r="J7"/>
+      <x:c r="K7"/>
+      <x:c r="L7" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="I7"/>
+      <x:c r="M7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>scan_barcode_payload_kind</x:v>
+        <x:v>barcode_payload_kind</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>Payload type</x:v>
       </x:c>
-      <x:c r="D8"/>
-      <x:c r="E8"/>
+      <x:c r="D8" t="str">
+        <x:v>text or url.</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F8"/>
       <x:c r="G8"/>
-      <x:c r="H8" t="str">
+      <x:c r="H8"/>
+      <x:c r="I8"/>
+      <x:c r="J8"/>
+      <x:c r="K8"/>
+      <x:c r="L8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="I8"/>
+      <x:c r="M8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>scan_barcode_payload_url</x:v>
+        <x:v>barcode_payload_url</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>Payload URL</x:v>
       </x:c>
-      <x:c r="D9"/>
-      <x:c r="E9"/>
+      <x:c r="D9" t="str">
+        <x:v>Present only when the exact payload is a safe absolute HTTP/HTTPS URL.</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F9"/>
-      <x:c r="G9"/>
-      <x:c r="H9" t="str">
+      <x:c r="G9" t="str">
+        <x:v>${barcode_payload_kind} = 'url'</x:v>
+      </x:c>
+      <x:c r="H9"/>
+      <x:c r="I9"/>
+      <x:c r="J9"/>
+      <x:c r="K9"/>
+      <x:c r="L9" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="I9" t="str">
-        <x:v>${scan_barcode_payload_kind} = 'url'</x:v>
-      </x:c>
+      <x:c r="M9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>text</x:v>
+        <x:v>hidden</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>scan_barcode_scan_time_iso</x:v>
+        <x:v>barcode_payload_sha256</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>Scan time</x:v>
-      </x:c>
-      <x:c r="D10"/>
+        <x:v>Barcode payload SHA-256</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>SHA-256 of the exact decoded payload.</x:v>
+      </x:c>
       <x:c r="E10"/>
       <x:c r="F10"/>
       <x:c r="G10"/>
-      <x:c r="H10" t="str">
+      <x:c r="H10"/>
+      <x:c r="I10"/>
+      <x:c r="J10"/>
+      <x:c r="K10"/>
+      <x:c r="L10" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="I10"/>
+      <x:c r="M10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>text</x:v>
+        <x:v>hidden</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>scan_barcode_source</x:v>
+        <x:v>verification_evidence_format</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>Capture source</x:v>
-      </x:c>
-      <x:c r="D11"/>
+        <x:v>Verification evidence format</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Evidence recipe identifier.</x:v>
+      </x:c>
       <x:c r="E11"/>
       <x:c r="F11"/>
       <x:c r="G11"/>
-      <x:c r="H11" t="str">
+      <x:c r="H11"/>
+      <x:c r="I11"/>
+      <x:c r="J11"/>
+      <x:c r="K11"/>
+      <x:c r="L11" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="I11"/>
+      <x:c r="M11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
         <x:v>hidden</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>scan_barcode_payload_sha256</x:v>
-      </x:c>
-      <x:c r="C12"/>
-      <x:c r="D12"/>
+        <x:v>verification_evidence_hash</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Verification evidence hash</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Evidence hash for this payload.</x:v>
+      </x:c>
       <x:c r="E12"/>
       <x:c r="F12"/>
       <x:c r="G12"/>
       <x:c r="H12"/>
       <x:c r="I12"/>
+      <x:c r="J12"/>
+      <x:c r="K12"/>
+      <x:c r="L12" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>hidden</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>scan_verification_evidence_format</x:v>
-      </x:c>
-      <x:c r="C13"/>
-      <x:c r="D13"/>
-      <x:c r="E13"/>
+        <x:v>barcode_scan_time_iso</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Scan time</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>ISO-8601 capture time.</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F13"/>
       <x:c r="G13"/>
       <x:c r="H13"/>
       <x:c r="I13"/>
+      <x:c r="J13"/>
+      <x:c r="K13"/>
+      <x:c r="L13" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>hidden</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>scan_verification_evidence_hash</x:v>
-      </x:c>
-      <x:c r="C14"/>
-      <x:c r="D14"/>
-      <x:c r="E14"/>
+        <x:v>barcode_source</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Capture source</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Scanner/source identifier.</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F14"/>
       <x:c r="G14"/>
       <x:c r="H14"/>
       <x:c r="I14"/>
+      <x:c r="J14"/>
+      <x:c r="K14"/>
+      <x:c r="L14" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>hidden</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>scan_methodmesh_full_json</x:v>
-      </x:c>
-      <x:c r="C15"/>
-      <x:c r="D15"/>
-      <x:c r="E15"/>
+        <x:v>methodmesh_full_json</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>MethodMesh full JSON</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>Complete MethodMesh execution/audit payload returned for the handled roundtrip.</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F15"/>
       <x:c r="G15"/>
       <x:c r="H15"/>
       <x:c r="I15"/>
+      <x:c r="J15"/>
+      <x:c r="K15"/>
+      <x:c r="L15" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>note</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>barcode_summary</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>Scanned: ${scan_barcode_payload}</x:v>
-      </x:c>
+        <x:v>end_group</x:v>
+      </x:c>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
       <x:c r="D16"/>
       <x:c r="E16"/>
       <x:c r="F16"/>
       <x:c r="G16"/>
       <x:c r="H16"/>
-      <x:c r="I16" t="str">
-        <x:v>${scan_barcode_payload} != ''</x:v>
-      </x:c>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
+      <x:c r="K16"/>
+      <x:c r="L16"/>
+      <x:c r="M16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>end_group</x:v>
-      </x:c>
-      <x:c r="B17"/>
-      <x:c r="C17"/>
-      <x:c r="D17"/>
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>return_summary</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>MethodMesh return captured. Status: ${methodmesh_status}</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>Decoded payload: ${barcode_payload}</x:v>
+      </x:c>
       <x:c r="E17"/>
       <x:c r="F17"/>
-      <x:c r="G17"/>
+      <x:c r="G17" t="str">
+        <x:v>${barcode_payload} != ''</x:v>
+      </x:c>
       <x:c r="H17"/>
       <x:c r="I17"/>
+      <x:c r="J17"/>
+      <x:c r="K17"/>
+      <x:c r="L17"/>
+      <x:c r="M17"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -887,6 +1021,8 @@
       <x:c r="D1" s="3" t="str">
         <x:v>instance_name</x:v>
       </x:c>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
@@ -896,11 +1032,13 @@
         <x:v>barcode_scan</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>2026090703</x:v>
+        <x:v>2026091201</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>${scan_barcode_payload}</x:v>
-      </x:c>
+        <x:v>${barcode_payload}</x:v>
+      </x:c>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>